<commit_message>
upteded pmc report code
</commit_message>
<xml_diff>
--- a/static/download/Contractor_Report_2.xlsx
+++ b/static/download/Contractor_Report_2.xlsx
@@ -816,77 +816,43 @@
           <t>59485</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>bhaneri jaat</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>oht work</t>
-        </is>
-      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Bhaneri Jaat Village OHT work</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="n">
-        <v>45229</v>
-      </c>
+          <t>GST Release Note</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>832500</v>
-      </c>
-      <c r="H16" t="n">
-        <v>446786</v>
-      </c>
-      <c r="I16" t="n">
-        <v>385714</v>
-      </c>
-      <c r="J16" t="n">
         <v>69428.52</v>
       </c>
-      <c r="K16" t="n">
-        <v>455142.52</v>
-      </c>
-      <c r="L16" t="n">
-        <v>3857.14</v>
-      </c>
-      <c r="M16" t="n">
-        <v>19285.7</v>
-      </c>
-      <c r="N16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" t="n">
-        <v>38571.4</v>
-      </c>
-      <c r="P16" t="n">
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="n">
         <v>69428.52</v>
       </c>
-      <c r="Q16" t="n">
-        <v>0</v>
-      </c>
-      <c r="R16" t="n">
-        <v>324000</v>
-      </c>
-      <c r="S16" t="n">
-        <v>0</v>
-      </c>
-      <c r="T16" t="n">
-        <v>0</v>
-      </c>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr"/>
       <c r="U16" t="n">
-        <v>47673</v>
+        <v>69429</v>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>03-11-2023 NEFT/AXISP00440155778/RIUP23/3003/AADI SHAKTI CONSTR/PUNB0388500 47673.00</t>
+          <t>06-12-2023 NEFT/AXISP00450230173/RIUP23/3623/AADI SHAKTI CONSTR/PUNB0388500 69429.00</t>
         </is>
       </c>
     </row>
@@ -906,11 +872,11 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>69428.52</v>
+        <v>105199.56</v>
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
@@ -923,16 +889,16 @@
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="n">
-        <v>69428.52</v>
+        <v>105199.56</v>
       </c>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="n">
-        <v>69429</v>
+        <v>148500</v>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>06-12-2023 NEFT/AXISP00450230173/RIUP23/3623/AADI SHAKTI CONSTR/PUNB0388500 69429.00</t>
+          <t>25-01-2024 NEFT/AXISP00464983349/RIUP23/4470/AADI SHAKTI CONSTR/PUNB0388500  148500.00</t>
         </is>
       </c>
     </row>
@@ -958,48 +924,48 @@
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>45329</v>
+        <v>45229</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>999000</v>
+        <v>832500</v>
       </c>
       <c r="H18" t="n">
-        <v>414558</v>
+        <v>446786</v>
       </c>
       <c r="I18" t="n">
-        <v>584442</v>
+        <v>385714</v>
       </c>
       <c r="J18" t="n">
-        <v>105199.56</v>
+        <v>69428.52</v>
       </c>
       <c r="K18" t="n">
-        <v>689641.5600000001</v>
+        <v>455142.52</v>
       </c>
       <c r="L18" t="n">
-        <v>5844.42</v>
+        <v>3857.14</v>
       </c>
       <c r="M18" t="n">
-        <v>29222.1</v>
+        <v>19285.7</v>
       </c>
       <c r="N18" t="n">
         <v>0</v>
       </c>
       <c r="O18" t="n">
-        <v>0</v>
+        <v>38571.4</v>
       </c>
       <c r="P18" t="n">
-        <v>105199.56</v>
+        <v>69428.52</v>
       </c>
       <c r="Q18" t="n">
         <v>0</v>
       </c>
       <c r="R18" t="n">
-        <v>549375</v>
+        <v>324000</v>
       </c>
       <c r="S18" t="n">
         <v>0</v>
@@ -1008,11 +974,11 @@
         <v>0</v>
       </c>
       <c r="U18" t="n">
-        <v>198000</v>
+        <v>47673</v>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>09-11-2023 NEFT/AXISP00442541879/RIUP23/3167/AADI SHAKTI CONSTR/PUNB0388500 198000.00</t>
+          <t>03-11-2023 NEFT/AXISP00440155778/RIUP23/3003/AADI SHAKTI CONSTR/PUNB0388500 47673.00</t>
         </is>
       </c>
     </row>
@@ -1022,43 +988,77 @@
           <t>59485</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>bhaneri jaat</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>oht work</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>GST Release Note</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
+          <t>Bhaneri Jaat Village OHT work</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>45329</v>
+      </c>
       <c r="F19" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
       <c r="G19" t="n">
+        <v>999000</v>
+      </c>
+      <c r="H19" t="n">
+        <v>414558</v>
+      </c>
+      <c r="I19" t="n">
+        <v>584442</v>
+      </c>
+      <c r="J19" t="n">
         <v>105199.56</v>
       </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
+      <c r="K19" t="n">
+        <v>689641.5600000001</v>
+      </c>
+      <c r="L19" t="n">
+        <v>5844.42</v>
+      </c>
+      <c r="M19" t="n">
+        <v>29222.1</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="n">
+        <v>105199.56</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>0</v>
+      </c>
       <c r="R19" t="n">
-        <v>105199.56</v>
-      </c>
-      <c r="S19" t="inlineStr"/>
-      <c r="T19" t="inlineStr"/>
+        <v>549375</v>
+      </c>
+      <c r="S19" t="n">
+        <v>0</v>
+      </c>
+      <c r="T19" t="n">
+        <v>0</v>
+      </c>
       <c r="U19" t="n">
-        <v>148500</v>
+        <v>198000</v>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>25-01-2024 NEFT/AXISP00464983349/RIUP23/4470/AADI SHAKTI CONSTR/PUNB0388500  148500.00</t>
+          <t>09-11-2023 NEFT/AXISP00442541879/RIUP23/3167/AADI SHAKTI CONSTR/PUNB0388500 198000.00</t>
         </is>
       </c>
     </row>
@@ -1416,11 +1416,11 @@
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>18713</v>
+        <v>52151</v>
       </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
@@ -1433,16 +1433,16 @@
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="n">
-        <v>18713</v>
+        <v>52151</v>
       </c>
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr"/>
       <c r="U26" t="n">
-        <v>18713</v>
+        <v>99000</v>
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>06-12-2023 NEFT/AXISP00450230172/RIUP23/3624/AADI SHAKTI CONSTR/PUNB0388500 18713.00</t>
+          <t>19-08-2024 NEFT/AXISP00529670925/RIUP24/1489/AADI SHAKTI CONSTR/PUNB0388500 99000.00</t>
         </is>
       </c>
     </row>
@@ -1452,77 +1452,43 @@
           <t>59486</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>kasampur</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>50kl 12m staging oht work</t>
-        </is>
-      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Kasampur Village 50KL 12m Staging  OHT work</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="n">
-        <v>45478</v>
-      </c>
+          <t>GST Release Note</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>341250</v>
-      </c>
-      <c r="H27" t="n">
-        <v>51525</v>
-      </c>
-      <c r="I27" t="n">
-        <v>289725</v>
-      </c>
-      <c r="J27" t="n">
-        <v>52151</v>
-      </c>
-      <c r="K27" t="n">
-        <v>341876</v>
-      </c>
-      <c r="L27" t="n">
-        <v>2897</v>
-      </c>
-      <c r="M27" t="n">
-        <v>14486</v>
-      </c>
-      <c r="N27" t="n">
-        <v>0</v>
-      </c>
-      <c r="O27" t="n">
-        <v>0</v>
-      </c>
-      <c r="P27" t="n">
-        <v>52151</v>
-      </c>
-      <c r="Q27" t="n">
-        <v>0</v>
-      </c>
+        <v>18713</v>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
       <c r="R27" t="n">
-        <v>272342</v>
-      </c>
-      <c r="S27" t="n">
-        <v>0</v>
-      </c>
-      <c r="T27" t="n">
-        <v>0</v>
-      </c>
+        <v>18713</v>
+      </c>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr"/>
       <c r="U27" t="n">
-        <v>250000</v>
+        <v>18713</v>
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>31-07-2024 NEFT/AXISP00522988539/RIUP24/1118/AADI SHAKTI CONSTR/PUNB0388500 250000.00</t>
+          <t>06-12-2023 NEFT/AXISP00450230172/RIUP23/3624/AADI SHAKTI CONSTR/PUNB0388500 18713.00</t>
         </is>
       </c>
     </row>
@@ -1532,43 +1498,77 @@
           <t>59486</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>kasampur</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>50kl 12m staging oht work</t>
+        </is>
+      </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>GST Release Note</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr"/>
+          <t>Kasampur Village 50KL 12m Staging  OHT work</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>45478</v>
+      </c>
       <c r="F28" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
       <c r="G28" t="n">
+        <v>341250</v>
+      </c>
+      <c r="H28" t="n">
+        <v>51525</v>
+      </c>
+      <c r="I28" t="n">
+        <v>289725</v>
+      </c>
+      <c r="J28" t="n">
         <v>52151</v>
       </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
+      <c r="K28" t="n">
+        <v>341876</v>
+      </c>
+      <c r="L28" t="n">
+        <v>2897</v>
+      </c>
+      <c r="M28" t="n">
+        <v>14486</v>
+      </c>
+      <c r="N28" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" t="n">
+        <v>52151</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>0</v>
+      </c>
       <c r="R28" t="n">
-        <v>52151</v>
-      </c>
-      <c r="S28" t="inlineStr"/>
-      <c r="T28" t="inlineStr"/>
+        <v>272342</v>
+      </c>
+      <c r="S28" t="n">
+        <v>0</v>
+      </c>
+      <c r="T28" t="n">
+        <v>0</v>
+      </c>
       <c r="U28" t="n">
-        <v>99000</v>
+        <v>250000</v>
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>19-08-2024 NEFT/AXISP00529670925/RIUP24/1489/AADI SHAKTI CONSTR/PUNB0388500 99000.00</t>
+          <t>31-07-2024 NEFT/AXISP00522988539/RIUP24/1118/AADI SHAKTI CONSTR/PUNB0388500 250000.00</t>
         </is>
       </c>
     </row>
@@ -1800,75 +1800,43 @@
           <t>59487</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>bhikki mazra</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>50kl 14m staging oht work</t>
-        </is>
-      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Bhikki Mazra Village 50KL 14m Staging  OHT work</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="n">
-        <v>45369</v>
-      </c>
+          <t>GST Release Note</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>633750</v>
-      </c>
-      <c r="H33" t="n">
-        <v>80906</v>
-      </c>
-      <c r="I33" t="n">
-        <v>552844</v>
-      </c>
-      <c r="J33" t="n">
-        <v>99512</v>
-      </c>
-      <c r="K33" t="n">
-        <v>652356</v>
-      </c>
-      <c r="L33" t="n">
-        <v>5528</v>
-      </c>
-      <c r="M33" t="n">
-        <v>27642</v>
-      </c>
-      <c r="N33" t="n">
-        <v>0</v>
-      </c>
-      <c r="O33" t="n">
-        <v>0</v>
-      </c>
-      <c r="P33" t="n">
-        <v>99512</v>
-      </c>
+        <v>7984</v>
+      </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="n">
-        <v>519674</v>
-      </c>
-      <c r="S33" t="n">
-        <v>0</v>
-      </c>
-      <c r="T33" t="n">
-        <v>0</v>
-      </c>
+        <v>7984</v>
+      </c>
+      <c r="S33" t="inlineStr"/>
+      <c r="T33" t="inlineStr"/>
       <c r="U33" t="n">
-        <v>519674</v>
+        <v>495000</v>
       </c>
       <c r="V33" t="inlineStr">
         <is>
-          <t>22-03-2024 NEFT/AXISP00483290486/RIUP23/5233/AADI SHAKTI CONSTR/PUNB0388500 519674.00</t>
+          <t>30-10-2024 NEFT/AXISP00561389904/RIUP24/2360/AADI SHAKTI CONSTR/PUNB0388500 495000.00</t>
         </is>
       </c>
     </row>
@@ -1888,11 +1856,11 @@
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G34" t="n">
-        <v>99512</v>
+        <v>135584</v>
       </c>
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr"/>
@@ -1905,18 +1873,10 @@
       <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr"/>
       <c r="R34" t="n">
-        <v>99512</v>
+        <v>135584</v>
       </c>
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr"/>
-      <c r="U34" t="n">
-        <v>99512</v>
-      </c>
-      <c r="V34" t="inlineStr">
-        <is>
-          <t>16-05-2024 NEFT/AXISP00500630402/RIUP24/0351/AADI SHAKTI CONSTR/PUNB0388500 99512.00</t>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1924,75 +1884,43 @@
           <t>59487</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>bhikki mazra</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>50kl 14m staging oht work</t>
-        </is>
-      </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Bhikki Mazra Village 50KL 14m Staging  OHT work</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="n">
-        <v>45517</v>
-      </c>
+          <t>GST Release Note</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G35" t="n">
-        <v>253500</v>
-      </c>
-      <c r="H35" t="n">
-        <v>209143</v>
-      </c>
-      <c r="I35" t="n">
-        <v>44357</v>
-      </c>
-      <c r="J35" t="n">
-        <v>7984</v>
-      </c>
-      <c r="K35" t="n">
-        <v>52341</v>
-      </c>
-      <c r="L35" t="n">
-        <v>444</v>
-      </c>
-      <c r="M35" t="n">
-        <v>2218</v>
-      </c>
-      <c r="N35" t="n">
-        <v>0</v>
-      </c>
-      <c r="O35" t="n">
-        <v>0</v>
-      </c>
-      <c r="P35" t="n">
-        <v>7984</v>
-      </c>
+        <v>99512</v>
+      </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr"/>
       <c r="R35" t="n">
-        <v>41695</v>
-      </c>
-      <c r="S35" t="n">
-        <v>0</v>
-      </c>
-      <c r="T35" t="n">
-        <v>0</v>
-      </c>
+        <v>99512</v>
+      </c>
+      <c r="S35" t="inlineStr"/>
+      <c r="T35" t="inlineStr"/>
       <c r="U35" t="n">
-        <v>99000</v>
+        <v>99512</v>
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>20-08-2024 NEFT/AXISP00530112321/RIUP24/1506/AADI SHAKTI CONSTR/PUNB0388500 99000.00</t>
+          <t>16-05-2024 NEFT/AXISP00500630402/RIUP24/0351/AADI SHAKTI CONSTR/PUNB0388500 99512.00</t>
         </is>
       </c>
     </row>
@@ -2002,43 +1930,75 @@
           <t>59487</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr"/>
-      <c r="C36" t="inlineStr"/>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>bhikki mazra</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>50kl 14m staging oht work</t>
+        </is>
+      </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>GST Release Note</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr"/>
+          <t>Bhikki Mazra Village 50KL 14m Staging  OHT work</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="n">
+        <v>45369</v>
+      </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G36" t="n">
-        <v>7984</v>
-      </c>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
+        <v>633750</v>
+      </c>
+      <c r="H36" t="n">
+        <v>80906</v>
+      </c>
+      <c r="I36" t="n">
+        <v>552844</v>
+      </c>
+      <c r="J36" t="n">
+        <v>99512</v>
+      </c>
+      <c r="K36" t="n">
+        <v>652356</v>
+      </c>
+      <c r="L36" t="n">
+        <v>5528</v>
+      </c>
+      <c r="M36" t="n">
+        <v>27642</v>
+      </c>
+      <c r="N36" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" t="n">
+        <v>0</v>
+      </c>
+      <c r="P36" t="n">
+        <v>99512</v>
+      </c>
       <c r="Q36" t="inlineStr"/>
       <c r="R36" t="n">
-        <v>7984</v>
-      </c>
-      <c r="S36" t="inlineStr"/>
-      <c r="T36" t="inlineStr"/>
+        <v>519674</v>
+      </c>
+      <c r="S36" t="n">
+        <v>0</v>
+      </c>
+      <c r="T36" t="n">
+        <v>0</v>
+      </c>
       <c r="U36" t="n">
-        <v>495000</v>
+        <v>519674</v>
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>30-10-2024 NEFT/AXISP00561389904/RIUP24/2360/AADI SHAKTI CONSTR/PUNB0388500 495000.00</t>
+          <t>22-03-2024 NEFT/AXISP00483290486/RIUP23/5233/AADI SHAKTI CONSTR/PUNB0388500 519674.00</t>
         </is>
       </c>
     </row>
@@ -2064,33 +2024,33 @@
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>45587</v>
+        <v>45517</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G37" t="n">
-        <v>912600</v>
+        <v>253500</v>
       </c>
       <c r="H37" t="n">
-        <v>159353</v>
+        <v>209143</v>
       </c>
       <c r="I37" t="n">
-        <v>753247</v>
+        <v>44357</v>
       </c>
       <c r="J37" t="n">
-        <v>135584</v>
+        <v>7984</v>
       </c>
       <c r="K37" t="n">
-        <v>888831</v>
+        <v>52341</v>
       </c>
       <c r="L37" t="n">
-        <v>7532</v>
+        <v>444</v>
       </c>
       <c r="M37" t="n">
-        <v>37662</v>
+        <v>2218</v>
       </c>
       <c r="N37" t="n">
         <v>0</v>
@@ -2099,11 +2059,11 @@
         <v>0</v>
       </c>
       <c r="P37" t="n">
-        <v>135584</v>
+        <v>7984</v>
       </c>
       <c r="Q37" t="inlineStr"/>
       <c r="R37" t="n">
-        <v>708053</v>
+        <v>41695</v>
       </c>
       <c r="S37" t="n">
         <v>0</v>
@@ -2112,11 +2072,11 @@
         <v>0</v>
       </c>
       <c r="U37" t="n">
-        <v>200000</v>
+        <v>99000</v>
       </c>
       <c r="V37" t="inlineStr">
         <is>
-          <t>21-06-2025 NEFT/AXISP00681347820/RIUP25/0513/AADI SHAKTI CONSTR/PUNB0388500 200000.00</t>
+          <t>20-08-2024 NEFT/AXISP00530112321/RIUP24/1506/AADI SHAKTI CONSTR/PUNB0388500 99000.00</t>
         </is>
       </c>
     </row>
@@ -2126,37 +2086,77 @@
           <t>59487</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
-      <c r="C38" t="inlineStr"/>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>bhikki mazra</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>50kl 14m staging oht work</t>
+        </is>
+      </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>GST Release Note</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr"/>
+          <t>Bhikki Mazra Village 50KL 14m Staging  OHT work</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>45587</v>
+      </c>
       <c r="F38" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
       <c r="G38" t="n">
+        <v>912600</v>
+      </c>
+      <c r="H38" t="n">
+        <v>159353</v>
+      </c>
+      <c r="I38" t="n">
+        <v>753247</v>
+      </c>
+      <c r="J38" t="n">
         <v>135584</v>
       </c>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr"/>
+      <c r="K38" t="n">
+        <v>888831</v>
+      </c>
+      <c r="L38" t="n">
+        <v>7532</v>
+      </c>
+      <c r="M38" t="n">
+        <v>37662</v>
+      </c>
+      <c r="N38" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" t="n">
+        <v>0</v>
+      </c>
+      <c r="P38" t="n">
+        <v>135584</v>
+      </c>
       <c r="Q38" t="inlineStr"/>
       <c r="R38" t="n">
-        <v>135584</v>
-      </c>
-      <c r="S38" t="inlineStr"/>
-      <c r="T38" t="inlineStr"/>
+        <v>708053</v>
+      </c>
+      <c r="S38" t="n">
+        <v>0</v>
+      </c>
+      <c r="T38" t="n">
+        <v>0</v>
+      </c>
+      <c r="U38" t="n">
+        <v>200000</v>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>21-06-2025 NEFT/AXISP00681347820/RIUP25/0513/AADI SHAKTI CONSTR/PUNB0388500 200000.00</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">

</xml_diff>